<commit_message>
adatbázis dummy adatok átalakitva és manuál teszt doksi hozzaadva
</commit_message>
<xml_diff>
--- a/Tervezés/Adatbázis_terv_project/teszt_adatbázis.xlsx
+++ b/Tervezés/Adatbázis_terv_project/teszt_adatbázis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sipos Fruzsina\Desktop\Adatbázis_terv_project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NapiCsepp\Tervezés\Adatbázis_terv_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37826FAA-D878-4ECC-B8EF-1D2DB7A94282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B6C4A3E-CC85-43D5-AE75-F2876E856B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9DD33D07-6BC9-4DD3-863C-32A92E35CA31}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="56">
   <si>
     <t>username</t>
   </si>
@@ -68,9 +68,6 @@
     <t>hu</t>
   </si>
   <si>
-    <t>user</t>
-  </si>
-  <si>
     <t>admin</t>
   </si>
   <si>
@@ -80,9 +77,6 @@
     <t>xyzc</t>
   </si>
   <si>
-    <t>en</t>
-  </si>
-  <si>
     <t>abi</t>
   </si>
   <si>
@@ -92,27 +86,12 @@
     <t>jjkijs</t>
   </si>
   <si>
-    <t>Tasks</t>
-  </si>
-  <si>
     <t>type_id</t>
   </si>
   <si>
     <t>difficulty_id</t>
   </si>
   <si>
-    <t>Levinni a szemetet</t>
-  </si>
-  <si>
-    <t>Mosás</t>
-  </si>
-  <si>
-    <t>Angol tz tanulni</t>
-  </si>
-  <si>
-    <t>Munkaruha elökeszit</t>
-  </si>
-  <si>
     <t>Types</t>
   </si>
   <si>
@@ -137,18 +116,6 @@
     <t>nehéz</t>
   </si>
   <si>
-    <t>Habits</t>
-  </si>
-  <si>
-    <t>habit_name</t>
-  </si>
-  <si>
-    <t>habit_type_id</t>
-  </si>
-  <si>
-    <t>habit_difficulty_id</t>
-  </si>
-  <si>
     <t>2 liter víz</t>
   </si>
   <si>
@@ -182,21 +149,9 @@
     <t>Nyaralás</t>
   </si>
   <si>
-    <t>Users_Tasks</t>
-  </si>
-  <si>
     <t>user_id</t>
   </si>
   <si>
-    <t>task_id</t>
-  </si>
-  <si>
-    <t>Users_Habits</t>
-  </si>
-  <si>
-    <t>habit_id</t>
-  </si>
-  <si>
     <t>true 1</t>
   </si>
   <si>
@@ -212,37 +167,43 @@
     <t>Events</t>
   </si>
   <si>
-    <t>Users_Events</t>
-  </si>
-  <si>
-    <t>task_name</t>
-  </si>
-  <si>
-    <t>task_type_id</t>
-  </si>
-  <si>
-    <t>task_difficulty_id</t>
-  </si>
-  <si>
-    <t>task_achive</t>
-  </si>
-  <si>
     <t>házimunka</t>
   </si>
   <si>
     <t>szokás</t>
   </si>
   <si>
-    <t>habit_create_date</t>
-  </si>
-  <si>
     <t>event_id</t>
   </si>
   <si>
-    <t>task_day</t>
-  </si>
-  <si>
-    <t>habit_target_days</t>
+    <t>activity_start_date</t>
+  </si>
+  <si>
+    <t>activity_end_date</t>
+  </si>
+  <si>
+    <t>progress_counter</t>
+  </si>
+  <si>
+    <t>activity_achive</t>
+  </si>
+  <si>
+    <t>activity_difficulty_id</t>
+  </si>
+  <si>
+    <t>activity_type_id</t>
+  </si>
+  <si>
+    <t>activity_name</t>
+  </si>
+  <si>
+    <t>activity_id</t>
+  </si>
+  <si>
+    <t>Activities</t>
+  </si>
+  <si>
+    <t>moderator</t>
   </si>
 </sst>
 </file>
@@ -330,22 +291,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -685,22 +649,23 @@
   <dimension ref="A2:I38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -711,7 +676,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>0</v>
@@ -749,7 +714,7 @@
         <v>9</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="G4" s="3">
         <v>45660</v>
@@ -760,19 +725,19 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G5" s="3">
         <v>45658</v>
@@ -783,19 +748,19 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="E6" s="1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="G6" s="3">
         <v>45660</v>
@@ -803,42 +768,44 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
-      <c r="H9" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="I9" s="8"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="E10" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>26</v>
+        <v>46</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -846,25 +813,28 @@
         <v>1</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C11" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D11" s="1">
         <v>1</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>53</v>
+      <c r="E11" s="3">
+        <v>45689</v>
       </c>
       <c r="F11" s="3">
-        <v>45810</v>
-      </c>
-      <c r="H11" s="1">
-        <v>1</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>63</v>
+        <v>45689</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I11" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -872,25 +842,28 @@
         <v>2</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C12" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D12" s="1">
-        <v>1</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>54</v>
+        <v>2</v>
+      </c>
+      <c r="E12" s="3">
+        <v>45355</v>
       </c>
       <c r="F12" s="3">
-        <v>45912</v>
-      </c>
-      <c r="H12" s="1">
-        <v>2</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>27</v>
+        <v>45720</v>
+      </c>
+      <c r="G12" s="1">
+        <v>10</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I12" s="1">
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -898,25 +871,28 @@
         <v>3</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C13" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" s="1">
         <v>3</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>53</v>
+      <c r="E13" s="3">
+        <v>45932</v>
       </c>
       <c r="F13" s="3">
-        <v>45864</v>
-      </c>
-      <c r="H13" s="1">
-        <v>3</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>28</v>
+        <v>45932</v>
+      </c>
+      <c r="G13" s="1">
+        <v>30</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I13" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -924,373 +900,229 @@
         <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="1">
+        <v>4</v>
+      </c>
+      <c r="D14" s="1">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3">
+        <v>45809</v>
+      </c>
+      <c r="F14" s="3">
+        <v>45809</v>
+      </c>
+      <c r="G14" s="1">
+        <v>350</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I14" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="G18" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>1</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="3">
+        <v>45784</v>
+      </c>
+      <c r="D20" s="3">
+        <v>45784</v>
+      </c>
+      <c r="E20" s="9">
+        <v>2</v>
+      </c>
+      <c r="G20" s="1">
+        <v>1</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>2</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="3">
+        <v>45962</v>
+      </c>
+      <c r="D21" s="3">
+        <v>45962</v>
+      </c>
+      <c r="E21" s="1">
+        <v>2</v>
+      </c>
+      <c r="G21" s="1">
+        <v>2</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>3</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="3">
+        <v>45831</v>
+      </c>
+      <c r="D22" s="3">
+        <v>45838</v>
+      </c>
+      <c r="E22" s="1">
+        <v>3</v>
+      </c>
+      <c r="G22" s="1">
+        <v>3</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G23" s="1">
+        <v>4</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="8"/>
+      <c r="G24" s="1">
+        <v>5</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>1</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>2</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="1">
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
         <v>3</v>
       </c>
-      <c r="D14" s="1">
-        <v>2</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="3">
-        <v>45931</v>
-      </c>
-      <c r="H14" s="1">
-        <v>4</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="H15" s="1">
-        <v>5</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="I18" s="5"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>1</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="1">
-        <v>4</v>
-      </c>
-      <c r="D19" s="1">
-        <v>1</v>
-      </c>
-      <c r="E19" s="1">
-        <v>30</v>
-      </c>
-      <c r="F19" s="3">
-        <v>45689</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <v>2</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="1">
-        <v>4</v>
-      </c>
-      <c r="D20" s="1">
-        <v>2</v>
-      </c>
-      <c r="E20" s="1">
-        <v>21</v>
-      </c>
-      <c r="F20" s="3">
-        <v>45720</v>
-      </c>
-      <c r="H20" s="1">
-        <v>1</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>3</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21" s="1">
-        <v>4</v>
-      </c>
-      <c r="D21" s="1">
-        <v>3</v>
-      </c>
-      <c r="E21" s="1">
-        <v>365</v>
-      </c>
-      <c r="F21" s="3">
-        <v>45932</v>
-      </c>
-      <c r="H21" s="1">
-        <v>2</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <v>4</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" s="1">
-        <v>4</v>
-      </c>
-      <c r="D22" s="1">
-        <v>3</v>
-      </c>
-      <c r="E22" s="1">
-        <v>34</v>
-      </c>
-      <c r="F22" s="3">
-        <v>45809</v>
-      </c>
-      <c r="H22" s="1">
-        <v>3</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="F25" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="G25" s="6"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
-        <v>1</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C27" s="3">
-        <v>45784</v>
-      </c>
-      <c r="D27" s="3">
-        <v>45784</v>
-      </c>
-      <c r="F27" s="1">
-        <v>1</v>
-      </c>
-      <c r="G27" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
-        <v>2</v>
-      </c>
       <c r="B28" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C28" s="3">
-        <v>45962</v>
-      </c>
-      <c r="D28" s="3">
-        <v>45962</v>
-      </c>
-      <c r="F28" s="1">
-        <v>1</v>
-      </c>
-      <c r="G28" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
-        <v>3</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C29" s="3">
-        <v>45831</v>
-      </c>
-      <c r="D29" s="3">
-        <v>45838</v>
-      </c>
-      <c r="F29" s="1">
-        <v>1</v>
-      </c>
-      <c r="G29" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F30" s="1">
-        <v>3</v>
-      </c>
-      <c r="G30" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F31" s="1">
-        <v>3</v>
-      </c>
-      <c r="G31" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B32" s="6"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E33" s="6"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
-        <v>1</v>
-      </c>
-      <c r="B34" s="1">
-        <v>2</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <v>1</v>
-      </c>
-      <c r="B35" s="1">
-        <v>4</v>
-      </c>
-      <c r="D35" s="1">
-        <v>1</v>
-      </c>
-      <c r="E35" s="1">
-        <v>1</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
-        <v>1</v>
-      </c>
-      <c r="B36" s="1">
-        <v>3</v>
-      </c>
-      <c r="D36" s="1">
-        <v>1</v>
-      </c>
-      <c r="E36" s="1">
-        <v>2</v>
-      </c>
+      <c r="A36" s="11"/>
+      <c r="B36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
-        <v>3</v>
-      </c>
-      <c r="B37" s="1">
-        <v>1</v>
-      </c>
-      <c r="D37" s="1">
-        <v>3</v>
-      </c>
-      <c r="E37" s="1">
-        <v>3</v>
-      </c>
+      <c r="A37" s="11"/>
+      <c r="B37" s="11"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
-        <v>3</v>
-      </c>
-      <c r="B38" s="1">
-        <v>3</v>
-      </c>
+      <c r="A38" s="11"/>
+      <c r="B38" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="D33:E33"/>
+  <mergeCells count="4">
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A9:I9"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{D3D6F310-829A-4E2B-A5EA-96D713F68F55}"/>

</xml_diff>